<commit_message>
DevLayer Academy - current stable version
</commit_message>
<xml_diff>
--- a/static/plantillas/plantilla_preguntas.xlsx
+++ b/static/plantillas/plantilla_preguntas.xlsx
@@ -2,7 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preguntas" sheetId="1" r:id="R21e8d0bb3fe4430b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preguntas" sheetId="1" r:id="Rd5f96ca3e2ae4c62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="R1c59063e1da046fa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20,23 +21,23 @@
     </x:font>
     <x:font>
       <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
       <x:sz val="16"/>
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
-      <x:sz val="10"/>
-      <x:color rgb="FF344054"/>
-      <x:name val="Carlito"/>
-    </x:font>
-    <x:font>
       <x:b/>
-      <x:sz val="10"/>
-      <x:color rgb="FFFFFFFF"/>
+      <x:sz val="11"/>
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -45,17 +46,22 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF10182D"/>
+        <x:fgColor rgb="FF1458D6"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFEEF5FF"/>
+        <x:fgColor rgb="FF0F172A"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF1677FF"/>
+        <x:fgColor rgb="FFE8EEFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3CD"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -66,45 +72,69 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="21">
+  <x:cellXfs count="33">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left"/>
+      <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center"/>
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left"/>
+      <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center"/>
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -308,56 +338,386 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="48" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="28" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="28" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="28" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="38" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="26" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="26" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="26" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="26" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="48" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="34" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="6" t="str">
+        <x:v>pregunta</x:v>
+      </x:c>
+      <x:c r="B1" s="6" t="str">
+        <x:v>tipo</x:v>
+      </x:c>
+      <x:c r="C1" s="6" t="str">
+        <x:v>opcion_a</x:v>
+      </x:c>
+      <x:c r="D1" s="6" t="str">
+        <x:v>opcion_b</x:v>
+      </x:c>
+      <x:c r="E1" s="6" t="str">
+        <x:v>opcion_c</x:v>
+      </x:c>
+      <x:c r="F1" s="6" t="str">
+        <x:v>opcion_d</x:v>
+      </x:c>
+      <x:c r="G1" s="6" t="str">
+        <x:v>respuesta_correcta</x:v>
+      </x:c>
+      <x:c r="H1" s="6" t="str">
+        <x:v>explicacion</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="12" t="str"/>
+      <x:c r="B2" s="12" t="str"/>
+      <x:c r="C2" s="12" t="str"/>
+      <x:c r="D2" s="12" t="str"/>
+      <x:c r="E2" s="12" t="str"/>
+      <x:c r="F2" s="12" t="str"/>
+      <x:c r="G2" s="12" t="str"/>
+      <x:c r="H2" s="12" t="str"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="12" t="str"/>
+      <x:c r="B3" s="12" t="str"/>
+      <x:c r="C3" s="12" t="str"/>
+      <x:c r="D3" s="12" t="str"/>
+      <x:c r="E3" s="12" t="str"/>
+      <x:c r="F3" s="12" t="str"/>
+      <x:c r="G3" s="12" t="str"/>
+      <x:c r="H3" s="12" t="str"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="12" t="str"/>
+      <x:c r="B4" s="12" t="str"/>
+      <x:c r="C4" s="12" t="str"/>
+      <x:c r="D4" s="12" t="str"/>
+      <x:c r="E4" s="12" t="str"/>
+      <x:c r="F4" s="12" t="str"/>
+      <x:c r="G4" s="12" t="str"/>
+      <x:c r="H4" s="12" t="str"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="12" t="str"/>
+      <x:c r="B5" s="12" t="str"/>
+      <x:c r="C5" s="12" t="str"/>
+      <x:c r="D5" s="12" t="str"/>
+      <x:c r="E5" s="12" t="str"/>
+      <x:c r="F5" s="12" t="str"/>
+      <x:c r="G5" s="12" t="str"/>
+      <x:c r="H5" s="12" t="str"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="12" t="str"/>
+      <x:c r="B6" s="12" t="str"/>
+      <x:c r="C6" s="12" t="str"/>
+      <x:c r="D6" s="12" t="str"/>
+      <x:c r="E6" s="12" t="str"/>
+      <x:c r="F6" s="12" t="str"/>
+      <x:c r="G6" s="12" t="str"/>
+      <x:c r="H6" s="12" t="str"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="12" t="str"/>
+      <x:c r="B7" s="12" t="str"/>
+      <x:c r="C7" s="12" t="str"/>
+      <x:c r="D7" s="12" t="str"/>
+      <x:c r="E7" s="12" t="str"/>
+      <x:c r="F7" s="12" t="str"/>
+      <x:c r="G7" s="12" t="str"/>
+      <x:c r="H7" s="12" t="str"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="12" t="str"/>
+      <x:c r="B8" s="12" t="str"/>
+      <x:c r="C8" s="12" t="str"/>
+      <x:c r="D8" s="12" t="str"/>
+      <x:c r="E8" s="12" t="str"/>
+      <x:c r="F8" s="12" t="str"/>
+      <x:c r="G8" s="12" t="str"/>
+      <x:c r="H8" s="12" t="str"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="12" t="str"/>
+      <x:c r="B9" s="12" t="str"/>
+      <x:c r="C9" s="12" t="str"/>
+      <x:c r="D9" s="12" t="str"/>
+      <x:c r="E9" s="12" t="str"/>
+      <x:c r="F9" s="12" t="str"/>
+      <x:c r="G9" s="12" t="str"/>
+      <x:c r="H9" s="12" t="str"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="12" t="str"/>
+      <x:c r="B10" s="12" t="str"/>
+      <x:c r="C10" s="12" t="str"/>
+      <x:c r="D10" s="12" t="str"/>
+      <x:c r="E10" s="12" t="str"/>
+      <x:c r="F10" s="12" t="str"/>
+      <x:c r="G10" s="12" t="str"/>
+      <x:c r="H10" s="12" t="str"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="12" t="str"/>
+      <x:c r="B11" s="12" t="str"/>
+      <x:c r="C11" s="12" t="str"/>
+      <x:c r="D11" s="12" t="str"/>
+      <x:c r="E11" s="12" t="str"/>
+      <x:c r="F11" s="12" t="str"/>
+      <x:c r="G11" s="12" t="str"/>
+      <x:c r="H11" s="12" t="str"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="12" t="str"/>
+      <x:c r="B12" s="12" t="str"/>
+      <x:c r="C12" s="12" t="str"/>
+      <x:c r="D12" s="12" t="str"/>
+      <x:c r="E12" s="12" t="str"/>
+      <x:c r="F12" s="12" t="str"/>
+      <x:c r="G12" s="12" t="str"/>
+      <x:c r="H12" s="12" t="str"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="12" t="str"/>
+      <x:c r="B13" s="12" t="str"/>
+      <x:c r="C13" s="12" t="str"/>
+      <x:c r="D13" s="12" t="str"/>
+      <x:c r="E13" s="12" t="str"/>
+      <x:c r="F13" s="12" t="str"/>
+      <x:c r="G13" s="12" t="str"/>
+      <x:c r="H13" s="12" t="str"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="12" t="str"/>
+      <x:c r="B14" s="12" t="str"/>
+      <x:c r="C14" s="12" t="str"/>
+      <x:c r="D14" s="12" t="str"/>
+      <x:c r="E14" s="12" t="str"/>
+      <x:c r="F14" s="12" t="str"/>
+      <x:c r="G14" s="12" t="str"/>
+      <x:c r="H14" s="12" t="str"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="12" t="str"/>
+      <x:c r="B15" s="12" t="str"/>
+      <x:c r="C15" s="12" t="str"/>
+      <x:c r="D15" s="12" t="str"/>
+      <x:c r="E15" s="12" t="str"/>
+      <x:c r="F15" s="12" t="str"/>
+      <x:c r="G15" s="12" t="str"/>
+      <x:c r="H15" s="12" t="str"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="12" t="str"/>
+      <x:c r="B16" s="12" t="str"/>
+      <x:c r="C16" s="12" t="str"/>
+      <x:c r="D16" s="12" t="str"/>
+      <x:c r="E16" s="12" t="str"/>
+      <x:c r="F16" s="12" t="str"/>
+      <x:c r="G16" s="12" t="str"/>
+      <x:c r="H16" s="12" t="str"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="12" t="str"/>
+      <x:c r="B17" s="12" t="str"/>
+      <x:c r="C17" s="12" t="str"/>
+      <x:c r="D17" s="12" t="str"/>
+      <x:c r="E17" s="12" t="str"/>
+      <x:c r="F17" s="12" t="str"/>
+      <x:c r="G17" s="12" t="str"/>
+      <x:c r="H17" s="12" t="str"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="12" t="str"/>
+      <x:c r="B18" s="12" t="str"/>
+      <x:c r="C18" s="12" t="str"/>
+      <x:c r="D18" s="12" t="str"/>
+      <x:c r="E18" s="12" t="str"/>
+      <x:c r="F18" s="12" t="str"/>
+      <x:c r="G18" s="12" t="str"/>
+      <x:c r="H18" s="12" t="str"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="12" t="str"/>
+      <x:c r="B19" s="12" t="str"/>
+      <x:c r="C19" s="12" t="str"/>
+      <x:c r="D19" s="12" t="str"/>
+      <x:c r="E19" s="12" t="str"/>
+      <x:c r="F19" s="12" t="str"/>
+      <x:c r="G19" s="12" t="str"/>
+      <x:c r="H19" s="12" t="str"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="12" t="str"/>
+      <x:c r="B20" s="12" t="str"/>
+      <x:c r="C20" s="12" t="str"/>
+      <x:c r="D20" s="12" t="str"/>
+      <x:c r="E20" s="12" t="str"/>
+      <x:c r="F20" s="12" t="str"/>
+      <x:c r="G20" s="12" t="str"/>
+      <x:c r="H20" s="12" t="str"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="12" t="str"/>
+      <x:c r="B21" s="12" t="str"/>
+      <x:c r="C21" s="12" t="str"/>
+      <x:c r="D21" s="12" t="str"/>
+      <x:c r="E21" s="12" t="str"/>
+      <x:c r="F21" s="12" t="str"/>
+      <x:c r="G21" s="12" t="str"/>
+      <x:c r="H21" s="12" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="B2:B21">
+      <x:formula1>"unica,multiple"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="40" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="30" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="42" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="5" t="str">
-        <x:v>Devlayer Academy · Plantilla de preguntas</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="34" customHeight="1">
-      <x:c r="A2" s="12" t="str">
-        <x:v>Previsualiza el XLSX antes de importar. El archivo no se almacena. Usa: unica, multiple, verdadero_falso o abierta.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="28" customHeight="1">
-      <x:c r="A4" s="20" t="str">
+      <x:c r="A1" s="17" t="str">
+        <x:v>Plantilla de cuestionarios automáticos</x:v>
+      </x:c>
+      <x:c r="B1" s="17"/>
+      <x:c r="C1" s="17"/>
+      <x:c r="D1" s="17"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="24" t="str">
+        <x:v>Campo</x:v>
+      </x:c>
+      <x:c r="B3" s="24" t="str">
+        <x:v>Qué colocar</x:v>
+      </x:c>
+      <x:c r="C3" s="24" t="str">
+        <x:v>Ejemplo</x:v>
+      </x:c>
+      <x:c r="D3" s="24" t="str">
+        <x:v>Regla</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="12" t="str">
         <x:v>pregunta</x:v>
       </x:c>
-      <x:c r="B4" s="20" t="str">
+      <x:c r="B4" s="12" t="str">
+        <x:v>Texto de la pregunta</x:v>
+      </x:c>
+      <x:c r="C4" s="12" t="str">
+        <x:v>Selecciona señales de confianza</x:v>
+      </x:c>
+      <x:c r="D4" s="12" t="str">
+        <x:v>Obligatorio</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="12" t="str">
         <x:v>tipo</x:v>
       </x:c>
-      <x:c r="C4" s="20" t="str">
-        <x:v>opcion_a</x:v>
-      </x:c>
-      <x:c r="D4" s="20" t="str">
-        <x:v>opcion_b</x:v>
-      </x:c>
-      <x:c r="E4" s="20" t="str">
-        <x:v>opcion_c</x:v>
-      </x:c>
-      <x:c r="F4" s="20" t="str">
-        <x:v>opcion_d</x:v>
-      </x:c>
-      <x:c r="G4" s="20" t="str">
+      <x:c r="B5" s="12" t="str">
+        <x:v>unica o multiple</x:v>
+      </x:c>
+      <x:c r="C5" s="12" t="str">
+        <x:v>multiple</x:v>
+      </x:c>
+      <x:c r="D5" s="12" t="str">
+        <x:v>No se aceptan abiertas ni verdadero/falso</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="12" t="str">
+        <x:v>opcion_a ... opcion_d</x:v>
+      </x:c>
+      <x:c r="B6" s="12" t="str">
+        <x:v>De 2 a 4 respuestas</x:v>
+      </x:c>
+      <x:c r="C6" s="12" t="str">
+        <x:v>Políticas claras</x:v>
+      </x:c>
+      <x:c r="D6" s="12" t="str">
+        <x:v>Obligatorio mínimo 2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="12" t="str">
         <x:v>respuesta_correcta</x:v>
       </x:c>
-      <x:c r="H4" s="20" t="str">
+      <x:c r="B7" s="12" t="str">
+        <x:v>Letras correctas</x:v>
+      </x:c>
+      <x:c r="C7" s="12" t="str">
+        <x:v>A o A,C</x:v>
+      </x:c>
+      <x:c r="D7" s="12" t="str">
+        <x:v>unica = 1 letra; multiple = 2 o más</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="12" t="str">
         <x:v>explicacion</x:v>
       </x:c>
+      <x:c r="B8" s="12" t="str">
+        <x:v>Retroalimentación opcional</x:v>
+      </x:c>
+      <x:c r="C8" s="12" t="str">
+        <x:v>La confianza reduce fricción</x:v>
+      </x:c>
+      <x:c r="D8" s="12" t="str">
+        <x:v>Opcional</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="32" t="str">
+        <x:v>IMPORTANTE</x:v>
+      </x:c>
+      <x:c r="B10" s="32"/>
+      <x:c r="C10" s="32"/>
+      <x:c r="D10" s="32"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="12" t="str">
+        <x:v>Selección única</x:v>
+      </x:c>
+      <x:c r="B11" s="12" t="str">
+        <x:v>respuesta_correcta = A</x:v>
+      </x:c>
+      <x:c r="C11" s="12"/>
+      <x:c r="D11" s="12"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="12" t="str">
+        <x:v>Varias selecciones</x:v>
+      </x:c>
+      <x:c r="B12" s="12" t="str">
+        <x:v>respuesta_correcta = A,C o A,B,D</x:v>
+      </x:c>
+      <x:c r="C12" s="12"/>
+      <x:c r="D12" s="12"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:H1"/>
-    <x:mergeCell ref="A2:H2"/>
+    <x:mergeCell ref="A1:D1"/>
+    <x:mergeCell ref="A10:D10"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>